<commit_message>
- Se incluyó un genérico Pad_value para cambiar el valor del padding rápidamente en el Registro_paralelo_serie.
</commit_message>
<xml_diff>
--- a/Operaciones prueba y combinaciones de valores de máquinas de estado.xlsx
+++ b/Operaciones prueba y combinaciones de valores de máquinas de estado.xlsx
@@ -1,18 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VivadoProjects\Convolution_v2\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FF40E1E-461E-4BF0-AB2A-139960722FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="10400"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Operaciones" sheetId="1" r:id="rId1"/>
     <sheet name="Combinaciones Valid_Data" sheetId="2" r:id="rId2"/>
-    <sheet name="Combinaciones Control_Bus_Out" sheetId="4" r:id="rId3"/>
+    <sheet name="Hoja1" sheetId="5" r:id="rId3"/>
+    <sheet name="Combinaciones Control_Bus_Out" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Combinaciones Control_Bus_Out'!$A$1:$F$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Combinaciones Control_Bus_Out'!$A$1:$F$181</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,31 +39,31 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <charset val="134"/>
+            <family val="2"/>
           </rPr>
           <t>TRUNC((BUS_VALID+2*PADDING-KERNEL)/STRIDE)+1-3
 Trunca la división como el operador / de enteros en VHDL.</t>
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0">
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <charset val="134"/>
+            <family val="2"/>
           </rPr>
           <t>Misma fórmula sin truncar la división (división real de Excel).</t>
         </r>
@@ -67,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="31">
   <si>
     <t>0,5,4,3,2,1,5,4,3,0,2,1,5,4,3,2,1,5,4,3,2,1,5,4,3,2,1</t>
   </si>
@@ -158,18 +165,15 @@
   <si>
     <t>Si X se declara natural/unsigned, el caso X = -1 (BUS_VALID=8, KERNEL=5, PADDING=0, STRIDE=3) no cabe.</t>
   </si>
+  <si>
+    <t>✓</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="28">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,196 +185,54 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <charset val="134"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -395,194 +257,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -614,274 +290,32 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -899,61 +333,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Coma" xfId="1" builtinId="3"/>
-    <cellStyle name="Moneda" xfId="2" builtinId="4"/>
-    <cellStyle name="Porcentaje" xfId="3" builtinId="5"/>
-    <cellStyle name="Coma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Moneda [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hipervínculo" xfId="6" builtinId="8"/>
-    <cellStyle name="Hipervínculo visitado" xfId="7" builtinId="9"/>
-    <cellStyle name="Nota" xfId="8" builtinId="10"/>
-    <cellStyle name="Texto de advertencia" xfId="9" builtinId="11"/>
-    <cellStyle name="Título" xfId="10" builtinId="15"/>
-    <cellStyle name="Texto explicativo" xfId="11" builtinId="53"/>
-    <cellStyle name="Título 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Título 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Título 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Título 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Entrada" xfId="16" builtinId="20"/>
-    <cellStyle name="Salida" xfId="17" builtinId="21"/>
-    <cellStyle name="Cálculo" xfId="18" builtinId="22"/>
-    <cellStyle name="Celda de comprobación" xfId="19" builtinId="23"/>
-    <cellStyle name="Celda vinculada" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Correcto" xfId="22" builtinId="26"/>
-    <cellStyle name="Incorrecto" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutro" xfId="24" builtinId="28"/>
-    <cellStyle name="Énfasis1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Énfasis1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Énfasis1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Énfasis1" xfId="28" builtinId="32"/>
-    <cellStyle name="Énfasis2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Énfasis2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Énfasis2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Énfasis2" xfId="32" builtinId="36"/>
-    <cellStyle name="Énfasis3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Énfasis3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Énfasis3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Énfasis3" xfId="36" builtinId="40"/>
-    <cellStyle name="Énfasis4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Énfasis4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Énfasis4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Énfasis4" xfId="40" builtinId="44"/>
-    <cellStyle name="Énfasis5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Énfasis5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Énfasis5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Énfasis5" xfId="44" builtinId="48"/>
-    <cellStyle name="Énfasis6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Énfasis6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Énfasis6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Énfasis6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 2" xfId="49"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="20">
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
@@ -994,7 +399,6 @@
       <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
@@ -1003,31 +407,30 @@
     <dxf>
       <alignment horizontal="center" vertical="center"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="B4:E19" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B4:E19" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="B4:E19" totalsRowShown="0">
+  <autoFilter ref="B4:E19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" name="BUS_VALID" dataDxfId="0"/>
-    <tableColumn id="2" name="PADDING" dataDxfId="1"/>
-    <tableColumn id="3" name="N" dataDxfId="2">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="BUS_VALID" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="PADDING" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="N" dataDxfId="17">
       <calculatedColumnFormula>B5+C5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" name="X" dataDxfId="3">
-      <calculatedColumnFormula>Tabla1[[#This Row],[N]]-5</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="X" dataDxfId="0">
+      <calculatedColumnFormula>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1035,12 +438,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabla2" displayName="Tabla2" ref="G4:I64" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="G4:I64" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla2" displayName="Tabla2" ref="G4:I64" totalsRowShown="0">
+  <autoFilter ref="G4:I64" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" name="N" dataDxfId="4"/>
-    <tableColumn id="2" name="KERNEL" dataDxfId="5"/>
-    <tableColumn id="3" name="Y" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="N" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="KERNEL" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Y" dataDxfId="14">
       <calculatedColumnFormula>G5-2*H5+7</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1049,11 +452,11 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabla3" displayName="Tabla3" ref="K4:L19" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="K4:L19" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabla3" displayName="Tabla3" ref="K4:L19" totalsRowShown="0">
+  <autoFilter ref="K4:L19" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="N" dataDxfId="7"/>
-    <tableColumn id="2" name="X" dataDxfId="8">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="N" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="X" dataDxfId="12">
       <calculatedColumnFormula>(K5/2)-2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1062,12 +465,12 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Tabla4" displayName="Tabla4" ref="O4:Q64" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="O4:Q64" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabla4" displayName="Tabla4" ref="O4:Q64" totalsRowShown="0">
+  <autoFilter ref="O4:Q64" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" name="N" dataDxfId="9"/>
-    <tableColumn id="2" name="KERNEL" dataDxfId="10"/>
-    <tableColumn id="3" name="Y" dataDxfId="11">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="N" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="KERNEL" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Y" dataDxfId="9">
       <calculatedColumnFormula>(O5-2*P5+7)/2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1076,11 +479,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Tabla36" displayName="Tabla36" ref="S4:T19" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="S4:T19" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabla36" displayName="Tabla36" ref="S4:T19" totalsRowShown="0">
+  <autoFilter ref="S4:T19" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="N" dataDxfId="12"/>
-    <tableColumn id="2" name="X" dataDxfId="13">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="N" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="X" dataDxfId="7">
       <calculatedColumnFormula>(Tabla36[[#This Row],[N]]/3)-1</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1089,14 +492,26 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Tabla47" displayName="Tabla47" ref="W4:Y64" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="W4:Y64" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Tabla47" displayName="Tabla47" ref="W4:Y64" totalsRowShown="0">
+  <autoFilter ref="W4:Y64" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" name="N" dataDxfId="14"/>
-    <tableColumn id="2" name="KERNEL" dataDxfId="15"/>
-    <tableColumn id="3" name="Y" dataDxfId="16">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="N" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="KERNEL" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Y" dataDxfId="4">
       <calculatedColumnFormula>(W5-2*X5+7)/3</calculatedColumnFormula>
     </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6B4087B-21AD-4435-8C5C-714DE90C9AD4}" name="Tabla28" displayName="Tabla28" ref="G4:I64" totalsRowShown="0">
+  <autoFilter ref="G4:I64" xr:uid="{B6B4087B-21AD-4435-8C5C-714DE90C9AD4}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{0B915746-E085-406A-BA0A-3136A357A3C9}" name="N" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{EA25C831-BC07-473A-9062-48AE0A731866}" name="KERNEL" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{1A28954D-B823-4207-A90A-D13B64E9B8A1}" name="Y" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1374,25 +789,25 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="C8:D12"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" outlineLevelCol="3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="65.8181818181818" customWidth="1"/>
-    <col min="8" max="8" width="42.7818181818182" customWidth="1"/>
+    <col min="4" max="4" width="65.77734375" customWidth="1"/>
+    <col min="8" max="8" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="4:4">
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D8" s="13" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="3:4">
+    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" s="15" t="s">
         <v>1</v>
       </c>
@@ -1400,7 +815,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="3:4">
+    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" s="15" t="s">
         <v>3</v>
       </c>
@@ -1408,13 +823,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="4:4">
+    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D11">
         <f>15+8+3</f>
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="4:4">
+    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D12">
         <f>D11*5</f>
         <v>130</v>
@@ -1422,63 +837,65 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Y64"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.8909090909091" style="13" customWidth="1"/>
-    <col min="3" max="3" width="13.7818181818182" style="13" customWidth="1"/>
-    <col min="4" max="5" width="7.33636363636364" style="13" customWidth="1"/>
-    <col min="7" max="9" width="11.5545454545455" style="13"/>
-    <col min="17" max="17" width="11.5545454545455" style="13"/>
-    <col min="25" max="25" width="11.5545454545455" style="13"/>
+    <col min="2" max="2" width="16.88671875" style="13" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="7.33203125" style="13" customWidth="1"/>
+    <col min="7" max="7" width="11.5546875" style="13"/>
+    <col min="8" max="8" width="13.21875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" style="13"/>
+    <col min="16" max="16" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5546875" style="13"/>
+    <col min="24" max="24" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5546875" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" s="12" customFormat="1" spans="1:1">
+    <row r="1" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="2:25">
-      <c r="B3" s="14" t="s">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="B3" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
       <c r="E3" s="14"/>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="K3" s="14" t="s">
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="K3" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="O3" s="14" t="s">
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="O3" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="S3" s="14" t="s">
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="S3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="W3" s="14" t="s">
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="W3" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="X3" s="14"/>
-      <c r="Y3" s="14"/>
-    </row>
-    <row r="4" spans="2:25">
+      <c r="X3" s="19"/>
+      <c r="Y3" s="19"/>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B4" s="13" t="s">
         <v>11</v>
       </c>
@@ -1531,7 +948,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="2:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B5" s="13">
         <v>128</v>
       </c>
@@ -1543,8 +960,8 @@
         <v>128</v>
       </c>
       <c r="E5" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>123</v>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>122</v>
       </c>
       <c r="G5" s="13">
         <v>128</v>
@@ -1578,7 +995,7 @@
       </c>
       <c r="T5" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>41.6666666666667</v>
+        <v>41.666666666666664</v>
       </c>
       <c r="W5" s="13">
         <v>128</v>
@@ -1588,10 +1005,10 @@
       </c>
       <c r="Y5" s="13">
         <f t="shared" ref="Y5:Y36" si="0">(W5-2*X5+7)/3</f>
-        <v>43.6666666666667</v>
-      </c>
-    </row>
-    <row r="6" spans="2:25">
+        <v>43.666666666666664</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B6" s="13">
         <v>128</v>
       </c>
@@ -1603,7 +1020,7 @@
         <v>129</v>
       </c>
       <c r="E6" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
         <v>124</v>
       </c>
       <c r="G6" s="13">
@@ -1651,7 +1068,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="2:25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B7" s="13">
         <v>128</v>
       </c>
@@ -1663,8 +1080,11 @@
         <v>130</v>
       </c>
       <c r="E7" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>125</v>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>126</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
       </c>
       <c r="G7" s="13">
         <v>128</v>
@@ -1698,7 +1118,7 @@
       </c>
       <c r="T7" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>42.3333333333333</v>
+        <v>42.333333333333336</v>
       </c>
       <c r="W7" s="13">
         <v>128</v>
@@ -1708,10 +1128,10 @@
       </c>
       <c r="Y7" s="13">
         <f t="shared" si="0"/>
-        <v>42.3333333333333</v>
-      </c>
-    </row>
-    <row r="8" spans="2:25">
+        <v>42.333333333333336</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" ht="15" x14ac:dyDescent="0.3">
       <c r="B8" s="13">
         <v>64</v>
       </c>
@@ -1723,8 +1143,8 @@
         <v>64</v>
       </c>
       <c r="E8" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>59</v>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>58</v>
       </c>
       <c r="G8" s="13">
         <v>128</v>
@@ -1735,6 +1155,9 @@
       <c r="I8" s="13">
         <f t="shared" si="2"/>
         <v>125</v>
+      </c>
+      <c r="J8" s="18" t="s">
+        <v>30</v>
       </c>
       <c r="K8" s="13">
         <v>64</v>
@@ -1758,7 +1181,7 @@
       </c>
       <c r="T8" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>20.3333333333333</v>
+        <v>20.333333333333332</v>
       </c>
       <c r="W8" s="13">
         <v>128</v>
@@ -1768,10 +1191,10 @@
       </c>
       <c r="Y8" s="13">
         <f t="shared" si="0"/>
-        <v>41.6666666666667</v>
-      </c>
-    </row>
-    <row r="9" spans="2:25">
+        <v>41.666666666666664</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B9" s="13">
         <v>64</v>
       </c>
@@ -1783,7 +1206,7 @@
         <v>65</v>
       </c>
       <c r="E9" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
         <v>60</v>
       </c>
       <c r="G9" s="13">
@@ -1818,7 +1241,7 @@
       </c>
       <c r="T9" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>20.6666666666667</v>
+        <v>20.666666666666668</v>
       </c>
       <c r="W9" s="13">
         <v>129</v>
@@ -1831,7 +1254,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="2:25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B10" s="13">
         <v>64</v>
       </c>
@@ -1843,8 +1266,8 @@
         <v>66</v>
       </c>
       <c r="E10" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>61</v>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>62</v>
       </c>
       <c r="G10" s="13">
         <v>129</v>
@@ -1888,10 +1311,10 @@
       </c>
       <c r="Y10" s="13">
         <f t="shared" si="0"/>
-        <v>43.3333333333333</v>
-      </c>
-    </row>
-    <row r="11" spans="2:25">
+        <v>43.333333333333336</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B11" s="13">
         <v>32</v>
       </c>
@@ -1903,8 +1326,8 @@
         <v>32</v>
       </c>
       <c r="E11" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>27</v>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>26</v>
       </c>
       <c r="F11" t="s">
         <v>17</v>
@@ -1941,7 +1364,7 @@
       </c>
       <c r="T11" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>9.66666666666667</v>
+        <v>9.6666666666666661</v>
       </c>
       <c r="W11" s="13">
         <v>129</v>
@@ -1951,10 +1374,10 @@
       </c>
       <c r="Y11" s="13">
         <f t="shared" si="0"/>
-        <v>42.6666666666667</v>
-      </c>
-    </row>
-    <row r="12" spans="2:25">
+        <v>42.666666666666664</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B12" s="13">
         <v>32</v>
       </c>
@@ -1966,7 +1389,7 @@
         <v>33</v>
       </c>
       <c r="E12" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
         <v>28</v>
       </c>
       <c r="G12" s="13">
@@ -2017,7 +1440,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="2:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B13" s="13">
         <v>32</v>
       </c>
@@ -2029,8 +1452,8 @@
         <v>34</v>
       </c>
       <c r="E13" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>29</v>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>30</v>
       </c>
       <c r="G13" s="13">
         <v>130</v>
@@ -2064,7 +1487,7 @@
       </c>
       <c r="T13" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>10.3333333333333</v>
+        <v>10.333333333333334</v>
       </c>
       <c r="W13" s="13">
         <v>130</v>
@@ -2074,10 +1497,10 @@
       </c>
       <c r="Y13" s="13">
         <f t="shared" si="0"/>
-        <v>44.3333333333333</v>
-      </c>
-    </row>
-    <row r="14" spans="2:25">
+        <v>44.333333333333336</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" ht="15" x14ac:dyDescent="0.3">
       <c r="B14" s="13">
         <v>16</v>
       </c>
@@ -2089,9 +1512,10 @@
         <v>16</v>
       </c>
       <c r="E14" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>11</v>
-      </c>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>10</v>
+      </c>
+      <c r="F14" s="17"/>
       <c r="G14" s="13">
         <v>130</v>
       </c>
@@ -2124,7 +1548,7 @@
       </c>
       <c r="T14" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>4.33333333333333</v>
+        <v>4.333333333333333</v>
       </c>
       <c r="W14" s="13">
         <v>130</v>
@@ -2134,10 +1558,10 @@
       </c>
       <c r="Y14" s="13">
         <f t="shared" si="0"/>
-        <v>43.6666666666667</v>
-      </c>
-    </row>
-    <row r="15" spans="2:25">
+        <v>43.666666666666664</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B15" s="13">
         <v>16</v>
       </c>
@@ -2149,7 +1573,7 @@
         <v>17</v>
       </c>
       <c r="E15" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
         <v>12</v>
       </c>
       <c r="G15" s="13">
@@ -2184,7 +1608,7 @@
       </c>
       <c r="T15" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>4.66666666666667</v>
+        <v>4.666666666666667</v>
       </c>
       <c r="W15" s="13">
         <v>130</v>
@@ -2197,7 +1621,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="2:25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B16" s="13">
         <v>16</v>
       </c>
@@ -2209,8 +1633,8 @@
         <v>18</v>
       </c>
       <c r="E16" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>13</v>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>14</v>
       </c>
       <c r="G16" s="13">
         <v>130</v>
@@ -2254,10 +1678,10 @@
       </c>
       <c r="Y16" s="13">
         <f t="shared" si="0"/>
-        <v>42.3333333333333</v>
-      </c>
-    </row>
-    <row r="17" spans="2:25">
+        <v>42.333333333333336</v>
+      </c>
+    </row>
+    <row r="17" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B17" s="13">
         <v>8</v>
       </c>
@@ -2269,8 +1693,8 @@
         <v>8</v>
       </c>
       <c r="E17" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>3</v>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>2</v>
       </c>
       <c r="G17" s="13">
         <v>64</v>
@@ -2304,7 +1728,7 @@
       </c>
       <c r="T17" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>1.66666666666667</v>
+        <v>1.6666666666666665</v>
       </c>
       <c r="W17" s="13">
         <v>64</v>
@@ -2314,10 +1738,10 @@
       </c>
       <c r="Y17" s="13">
         <f t="shared" si="0"/>
-        <v>22.3333333333333</v>
-      </c>
-    </row>
-    <row r="18" spans="2:25">
+        <v>22.333333333333332</v>
+      </c>
+    </row>
+    <row r="18" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B18" s="13">
         <v>8</v>
       </c>
@@ -2329,7 +1753,7 @@
         <v>9</v>
       </c>
       <c r="E18" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
         <v>4</v>
       </c>
       <c r="G18" s="13">
@@ -2374,10 +1798,10 @@
       </c>
       <c r="Y18" s="13">
         <f t="shared" si="0"/>
-        <v>21.6666666666667</v>
-      </c>
-    </row>
-    <row r="19" spans="2:25">
+        <v>21.666666666666668</v>
+      </c>
+    </row>
+    <row r="19" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B19" s="13">
         <v>8</v>
       </c>
@@ -2389,8 +1813,8 @@
         <v>10</v>
       </c>
       <c r="E19" s="13">
-        <f>Tabla1[[#This Row],[N]]-5</f>
-        <v>5</v>
+        <f>Tabla1[[#This Row],[N]]-6 + 1*Tabla1[[#This Row],[PADDING]]</f>
+        <v>6</v>
       </c>
       <c r="G19" s="13">
         <v>64</v>
@@ -2424,7 +1848,7 @@
       </c>
       <c r="T19" s="13">
         <f>(Tabla36[[#This Row],[N]]/3)-1</f>
-        <v>2.33333333333333</v>
+        <v>2.3333333333333335</v>
       </c>
       <c r="W19" s="13">
         <v>64</v>
@@ -2437,7 +1861,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="7:25">
+    <row r="20" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G20" s="13">
         <v>64</v>
       </c>
@@ -2466,10 +1890,10 @@
       </c>
       <c r="Y20" s="13">
         <f t="shared" si="0"/>
-        <v>20.3333333333333</v>
-      </c>
-    </row>
-    <row r="21" spans="7:25">
+        <v>20.333333333333332</v>
+      </c>
+    </row>
+    <row r="21" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G21" s="13">
         <v>65</v>
       </c>
@@ -2498,10 +1922,10 @@
       </c>
       <c r="Y21" s="13">
         <f t="shared" si="0"/>
-        <v>22.6666666666667</v>
-      </c>
-    </row>
-    <row r="22" spans="7:25">
+        <v>22.666666666666668</v>
+      </c>
+    </row>
+    <row r="22" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G22" s="13">
         <v>65</v>
       </c>
@@ -2536,9 +1960,18 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="3:25">
-      <c r="C23" s="13" t="s">
-        <v>17</v>
+    <row r="23" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B23" s="13">
+        <v>128</v>
+      </c>
+      <c r="C23" s="13">
+        <v>0</v>
+      </c>
+      <c r="D23" s="13">
+        <v>128</v>
+      </c>
+      <c r="E23" s="13">
+        <v>122</v>
       </c>
       <c r="G23" s="13">
         <v>65</v>
@@ -2568,10 +2001,22 @@
       </c>
       <c r="Y23" s="13">
         <f t="shared" si="0"/>
-        <v>21.3333333333333</v>
-      </c>
-    </row>
-    <row r="24" spans="7:25">
+        <v>21.333333333333332</v>
+      </c>
+    </row>
+    <row r="24" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B24" s="13">
+        <v>128</v>
+      </c>
+      <c r="C24" s="13">
+        <v>1</v>
+      </c>
+      <c r="D24" s="13">
+        <v>129</v>
+      </c>
+      <c r="E24" s="13">
+        <v>124</v>
+      </c>
       <c r="G24" s="13">
         <v>65</v>
       </c>
@@ -2600,10 +2045,22 @@
       </c>
       <c r="Y24" s="13">
         <f t="shared" si="0"/>
-        <v>20.6666666666667</v>
-      </c>
-    </row>
-    <row r="25" spans="7:25">
+        <v>20.666666666666668</v>
+      </c>
+    </row>
+    <row r="25" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B25" s="13">
+        <v>128</v>
+      </c>
+      <c r="C25" s="13">
+        <v>2</v>
+      </c>
+      <c r="D25" s="13">
+        <v>130</v>
+      </c>
+      <c r="E25" s="13">
+        <v>126</v>
+      </c>
       <c r="G25" s="13">
         <v>66</v>
       </c>
@@ -2635,7 +2092,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="7:25">
+    <row r="26" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G26" s="13">
         <v>66</v>
       </c>
@@ -2664,10 +2121,10 @@
       </c>
       <c r="Y26" s="13">
         <f t="shared" si="0"/>
-        <v>22.3333333333333</v>
-      </c>
-    </row>
-    <row r="27" spans="7:25">
+        <v>22.333333333333332</v>
+      </c>
+    </row>
+    <row r="27" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G27" s="13">
         <v>66</v>
       </c>
@@ -2696,10 +2153,10 @@
       </c>
       <c r="Y27" s="13">
         <f t="shared" si="0"/>
-        <v>21.6666666666667</v>
-      </c>
-    </row>
-    <row r="28" spans="7:25">
+        <v>21.666666666666668</v>
+      </c>
+    </row>
+    <row r="28" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G28" s="13">
         <v>66</v>
       </c>
@@ -2731,7 +2188,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="7:25">
+    <row r="29" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G29" s="13">
         <v>32</v>
       </c>
@@ -2760,10 +2217,10 @@
       </c>
       <c r="Y29" s="13">
         <f t="shared" si="0"/>
-        <v>11.6666666666667</v>
-      </c>
-    </row>
-    <row r="30" spans="7:25">
+        <v>11.666666666666666</v>
+      </c>
+    </row>
+    <row r="30" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G30" s="13">
         <v>32</v>
       </c>
@@ -2795,7 +2252,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="7:25">
+    <row r="31" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G31" s="13">
         <v>32</v>
       </c>
@@ -2824,10 +2281,10 @@
       </c>
       <c r="Y31" s="13">
         <f t="shared" si="0"/>
-        <v>10.3333333333333</v>
-      </c>
-    </row>
-    <row r="32" spans="7:25">
+        <v>10.333333333333334</v>
+      </c>
+    </row>
+    <row r="32" spans="2:25" x14ac:dyDescent="0.25">
       <c r="G32" s="13">
         <v>32</v>
       </c>
@@ -2856,10 +2313,10 @@
       </c>
       <c r="Y32" s="13">
         <f t="shared" si="0"/>
-        <v>9.66666666666667</v>
-      </c>
-    </row>
-    <row r="33" spans="7:25">
+        <v>9.6666666666666661</v>
+      </c>
+    </row>
+    <row r="33" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G33" s="13">
         <v>33</v>
       </c>
@@ -2891,7 +2348,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="7:25">
+    <row r="34" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G34" s="13">
         <v>33</v>
       </c>
@@ -2920,10 +2377,10 @@
       </c>
       <c r="Y34" s="13">
         <f t="shared" si="0"/>
-        <v>11.3333333333333</v>
-      </c>
-    </row>
-    <row r="35" spans="7:25">
+        <v>11.333333333333334</v>
+      </c>
+    </row>
+    <row r="35" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G35" s="13">
         <v>33</v>
       </c>
@@ -2952,10 +2409,10 @@
       </c>
       <c r="Y35" s="13">
         <f t="shared" si="0"/>
-        <v>10.6666666666667</v>
-      </c>
-    </row>
-    <row r="36" spans="7:25">
+        <v>10.666666666666666</v>
+      </c>
+    </row>
+    <row r="36" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G36" s="13">
         <v>33</v>
       </c>
@@ -2987,7 +2444,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="7:25">
+    <row r="37" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G37" s="13">
         <v>34</v>
       </c>
@@ -3016,10 +2473,10 @@
       </c>
       <c r="Y37" s="13">
         <f t="shared" ref="Y37:Y64" si="5">(W37-2*X37+7)/3</f>
-        <v>12.3333333333333</v>
-      </c>
-    </row>
-    <row r="38" spans="7:25">
+        <v>12.333333333333334</v>
+      </c>
+    </row>
+    <row r="38" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G38" s="13">
         <v>34</v>
       </c>
@@ -3048,10 +2505,10 @@
       </c>
       <c r="Y38" s="13">
         <f t="shared" si="5"/>
-        <v>11.6666666666667</v>
-      </c>
-    </row>
-    <row r="39" spans="7:25">
+        <v>11.666666666666666</v>
+      </c>
+    </row>
+    <row r="39" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G39" s="13">
         <v>34</v>
       </c>
@@ -3083,7 +2540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="7:25">
+    <row r="40" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G40" s="13">
         <v>34</v>
       </c>
@@ -3112,10 +2569,10 @@
       </c>
       <c r="Y40" s="13">
         <f t="shared" si="5"/>
-        <v>10.3333333333333</v>
-      </c>
-    </row>
-    <row r="41" spans="7:25">
+        <v>10.333333333333334</v>
+      </c>
+    </row>
+    <row r="41" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G41" s="13">
         <v>16</v>
       </c>
@@ -3144,10 +2601,10 @@
       </c>
       <c r="Y41" s="13">
         <f t="shared" si="5"/>
-        <v>6.33333333333333</v>
-      </c>
-    </row>
-    <row r="42" spans="7:25">
+        <v>6.333333333333333</v>
+      </c>
+    </row>
+    <row r="42" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G42" s="13">
         <v>16</v>
       </c>
@@ -3176,10 +2633,10 @@
       </c>
       <c r="Y42" s="13">
         <f t="shared" si="5"/>
-        <v>5.66666666666667</v>
-      </c>
-    </row>
-    <row r="43" spans="7:25">
+        <v>5.666666666666667</v>
+      </c>
+    </row>
+    <row r="43" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G43" s="13">
         <v>16</v>
       </c>
@@ -3211,7 +2668,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="7:25">
+    <row r="44" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G44" s="13">
         <v>16</v>
       </c>
@@ -3240,10 +2697,10 @@
       </c>
       <c r="Y44" s="13">
         <f t="shared" si="5"/>
-        <v>4.33333333333333</v>
-      </c>
-    </row>
-    <row r="45" spans="7:25">
+        <v>4.333333333333333</v>
+      </c>
+    </row>
+    <row r="45" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G45" s="13">
         <v>17</v>
       </c>
@@ -3272,10 +2729,10 @@
       </c>
       <c r="Y45" s="13">
         <f t="shared" si="5"/>
-        <v>6.66666666666667</v>
-      </c>
-    </row>
-    <row r="46" spans="7:25">
+        <v>6.666666666666667</v>
+      </c>
+    </row>
+    <row r="46" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G46" s="13">
         <v>17</v>
       </c>
@@ -3307,7 +2764,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="7:25">
+    <row r="47" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G47" s="13">
         <v>17</v>
       </c>
@@ -3336,10 +2793,10 @@
       </c>
       <c r="Y47" s="13">
         <f t="shared" si="5"/>
-        <v>5.33333333333333</v>
-      </c>
-    </row>
-    <row r="48" spans="7:25">
+        <v>5.333333333333333</v>
+      </c>
+    </row>
+    <row r="48" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G48" s="13">
         <v>17</v>
       </c>
@@ -3368,10 +2825,10 @@
       </c>
       <c r="Y48" s="13">
         <f t="shared" si="5"/>
-        <v>4.66666666666667</v>
-      </c>
-    </row>
-    <row r="49" spans="7:25">
+        <v>4.666666666666667</v>
+      </c>
+    </row>
+    <row r="49" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G49" s="13">
         <v>18</v>
       </c>
@@ -3403,7 +2860,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="7:25">
+    <row r="50" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G50" s="13">
         <v>18</v>
       </c>
@@ -3432,10 +2889,10 @@
       </c>
       <c r="Y50" s="13">
         <f t="shared" si="5"/>
-        <v>6.33333333333333</v>
-      </c>
-    </row>
-    <row r="51" spans="7:25">
+        <v>6.333333333333333</v>
+      </c>
+    </row>
+    <row r="51" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G51" s="13">
         <v>18</v>
       </c>
@@ -3464,10 +2921,10 @@
       </c>
       <c r="Y51" s="13">
         <f t="shared" si="5"/>
-        <v>5.66666666666667</v>
-      </c>
-    </row>
-    <row r="52" spans="7:25">
+        <v>5.666666666666667</v>
+      </c>
+    </row>
+    <row r="52" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G52" s="13">
         <v>18</v>
       </c>
@@ -3499,7 +2956,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="7:25">
+    <row r="53" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G53" s="13">
         <v>8</v>
       </c>
@@ -3528,10 +2985,10 @@
       </c>
       <c r="Y53" s="13">
         <f t="shared" si="5"/>
-        <v>3.66666666666667</v>
-      </c>
-    </row>
-    <row r="54" spans="7:25">
+        <v>3.6666666666666665</v>
+      </c>
+    </row>
+    <row r="54" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G54" s="13">
         <v>8</v>
       </c>
@@ -3563,7 +3020,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="7:25">
+    <row r="55" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G55" s="13">
         <v>8</v>
       </c>
@@ -3592,10 +3049,10 @@
       </c>
       <c r="Y55" s="13">
         <f t="shared" si="5"/>
-        <v>2.33333333333333</v>
-      </c>
-    </row>
-    <row r="56" spans="7:25">
+        <v>2.3333333333333335</v>
+      </c>
+    </row>
+    <row r="56" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G56" s="13">
         <v>8</v>
       </c>
@@ -3624,10 +3081,10 @@
       </c>
       <c r="Y56" s="13">
         <f t="shared" si="5"/>
-        <v>1.66666666666667</v>
-      </c>
-    </row>
-    <row r="57" spans="7:25">
+        <v>1.6666666666666667</v>
+      </c>
+    </row>
+    <row r="57" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G57" s="13">
         <v>9</v>
       </c>
@@ -3659,7 +3116,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="7:25">
+    <row r="58" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G58" s="13">
         <v>9</v>
       </c>
@@ -3688,10 +3145,10 @@
       </c>
       <c r="Y58" s="13">
         <f t="shared" si="5"/>
-        <v>3.33333333333333</v>
-      </c>
-    </row>
-    <row r="59" spans="7:25">
+        <v>3.3333333333333335</v>
+      </c>
+    </row>
+    <row r="59" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G59" s="13">
         <v>9</v>
       </c>
@@ -3720,10 +3177,10 @@
       </c>
       <c r="Y59" s="13">
         <f t="shared" si="5"/>
-        <v>2.66666666666667</v>
-      </c>
-    </row>
-    <row r="60" spans="7:25">
+        <v>2.6666666666666665</v>
+      </c>
+    </row>
+    <row r="60" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G60" s="13">
         <v>9</v>
       </c>
@@ -3755,7 +3212,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="7:25">
+    <row r="61" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G61" s="13">
         <v>10</v>
       </c>
@@ -3784,10 +3241,10 @@
       </c>
       <c r="Y61" s="13">
         <f t="shared" si="5"/>
-        <v>4.33333333333333</v>
-      </c>
-    </row>
-    <row r="62" spans="7:25">
+        <v>4.333333333333333</v>
+      </c>
+    </row>
+    <row r="62" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G62" s="13">
         <v>10</v>
       </c>
@@ -3816,10 +3273,10 @@
       </c>
       <c r="Y62" s="13">
         <f t="shared" si="5"/>
-        <v>3.66666666666667</v>
-      </c>
-    </row>
-    <row r="63" spans="7:25">
+        <v>3.6666666666666665</v>
+      </c>
+    </row>
+    <row r="63" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G63" s="13">
         <v>10</v>
       </c>
@@ -3851,7 +3308,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="64" spans="7:25">
+    <row r="64" spans="7:25" x14ac:dyDescent="0.25">
       <c r="G64" s="13">
         <v>10</v>
       </c>
@@ -3880,20 +3337,19 @@
       </c>
       <c r="Y64" s="13">
         <f t="shared" si="5"/>
-        <v>2.33333333333333</v>
+        <v>2.3333333333333335</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="W3:Y3"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="O3:Q3"/>
     <mergeCell ref="S3:U3"/>
-    <mergeCell ref="W3:Y3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="6">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
@@ -3906,22 +3362,595 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3FAE71D-CE45-4183-B4CF-C0DF84B83244}">
+  <dimension ref="G3:I64"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="3" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G3" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+    </row>
+    <row r="4" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G4" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G5" s="13">
+        <v>128</v>
+      </c>
+      <c r="H5" s="13">
+        <v>2</v>
+      </c>
+      <c r="I5" s="13"/>
+    </row>
+    <row r="6" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G6" s="13">
+        <v>128</v>
+      </c>
+      <c r="H6" s="13">
+        <v>3</v>
+      </c>
+      <c r="I6" s="13"/>
+    </row>
+    <row r="7" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G7" s="13">
+        <v>128</v>
+      </c>
+      <c r="H7" s="13">
+        <v>4</v>
+      </c>
+      <c r="I7" s="13"/>
+    </row>
+    <row r="8" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G8" s="13">
+        <v>128</v>
+      </c>
+      <c r="H8" s="13">
+        <v>5</v>
+      </c>
+      <c r="I8" s="13"/>
+    </row>
+    <row r="9" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G9" s="13">
+        <v>129</v>
+      </c>
+      <c r="H9" s="13">
+        <v>2</v>
+      </c>
+      <c r="I9" s="13"/>
+    </row>
+    <row r="10" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G10" s="13">
+        <v>129</v>
+      </c>
+      <c r="H10" s="13">
+        <v>3</v>
+      </c>
+      <c r="I10" s="13"/>
+    </row>
+    <row r="11" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G11" s="13">
+        <v>129</v>
+      </c>
+      <c r="H11" s="13">
+        <v>4</v>
+      </c>
+      <c r="I11" s="13"/>
+    </row>
+    <row r="12" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G12" s="13">
+        <v>129</v>
+      </c>
+      <c r="H12" s="13">
+        <v>5</v>
+      </c>
+      <c r="I12" s="13"/>
+    </row>
+    <row r="13" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G13" s="13">
+        <v>130</v>
+      </c>
+      <c r="H13" s="13">
+        <v>2</v>
+      </c>
+      <c r="I13" s="13"/>
+    </row>
+    <row r="14" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G14" s="13">
+        <v>130</v>
+      </c>
+      <c r="H14" s="13">
+        <v>3</v>
+      </c>
+      <c r="I14" s="13"/>
+    </row>
+    <row r="15" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G15" s="13">
+        <v>130</v>
+      </c>
+      <c r="H15" s="13">
+        <v>4</v>
+      </c>
+      <c r="I15" s="13"/>
+    </row>
+    <row r="16" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G16" s="13">
+        <v>130</v>
+      </c>
+      <c r="H16" s="13">
+        <v>5</v>
+      </c>
+      <c r="I16" s="13"/>
+    </row>
+    <row r="17" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G17" s="13">
+        <v>64</v>
+      </c>
+      <c r="H17" s="13">
+        <v>2</v>
+      </c>
+      <c r="I17" s="13"/>
+    </row>
+    <row r="18" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G18" s="13">
+        <v>64</v>
+      </c>
+      <c r="H18" s="13">
+        <v>3</v>
+      </c>
+      <c r="I18" s="13"/>
+    </row>
+    <row r="19" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G19" s="13">
+        <v>64</v>
+      </c>
+      <c r="H19" s="13">
+        <v>4</v>
+      </c>
+      <c r="I19" s="13"/>
+    </row>
+    <row r="20" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G20" s="13">
+        <v>64</v>
+      </c>
+      <c r="H20" s="13">
+        <v>5</v>
+      </c>
+      <c r="I20" s="13"/>
+    </row>
+    <row r="21" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G21" s="13">
+        <v>65</v>
+      </c>
+      <c r="H21" s="13">
+        <v>2</v>
+      </c>
+      <c r="I21" s="13"/>
+    </row>
+    <row r="22" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G22" s="13">
+        <v>65</v>
+      </c>
+      <c r="H22" s="13">
+        <v>3</v>
+      </c>
+      <c r="I22" s="13"/>
+    </row>
+    <row r="23" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G23" s="13">
+        <v>65</v>
+      </c>
+      <c r="H23" s="13">
+        <v>4</v>
+      </c>
+      <c r="I23" s="13"/>
+    </row>
+    <row r="24" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G24" s="13">
+        <v>65</v>
+      </c>
+      <c r="H24" s="13">
+        <v>5</v>
+      </c>
+      <c r="I24" s="13"/>
+    </row>
+    <row r="25" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G25" s="13">
+        <v>66</v>
+      </c>
+      <c r="H25" s="13">
+        <v>2</v>
+      </c>
+      <c r="I25" s="13"/>
+    </row>
+    <row r="26" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G26" s="13">
+        <v>66</v>
+      </c>
+      <c r="H26" s="13">
+        <v>3</v>
+      </c>
+      <c r="I26" s="13"/>
+    </row>
+    <row r="27" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G27" s="13">
+        <v>66</v>
+      </c>
+      <c r="H27" s="13">
+        <v>4</v>
+      </c>
+      <c r="I27" s="13"/>
+    </row>
+    <row r="28" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G28" s="13">
+        <v>66</v>
+      </c>
+      <c r="H28" s="13">
+        <v>5</v>
+      </c>
+      <c r="I28" s="13"/>
+    </row>
+    <row r="29" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G29" s="13">
+        <v>32</v>
+      </c>
+      <c r="H29" s="13">
+        <v>2</v>
+      </c>
+      <c r="I29" s="13"/>
+    </row>
+    <row r="30" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G30" s="13">
+        <v>32</v>
+      </c>
+      <c r="H30" s="13">
+        <v>3</v>
+      </c>
+      <c r="I30" s="13"/>
+    </row>
+    <row r="31" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G31" s="13">
+        <v>32</v>
+      </c>
+      <c r="H31" s="13">
+        <v>4</v>
+      </c>
+      <c r="I31" s="13"/>
+    </row>
+    <row r="32" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G32" s="13">
+        <v>32</v>
+      </c>
+      <c r="H32" s="13">
+        <v>5</v>
+      </c>
+      <c r="I32" s="13"/>
+    </row>
+    <row r="33" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G33" s="13">
+        <v>33</v>
+      </c>
+      <c r="H33" s="13">
+        <v>2</v>
+      </c>
+      <c r="I33" s="13"/>
+    </row>
+    <row r="34" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G34" s="13">
+        <v>33</v>
+      </c>
+      <c r="H34" s="13">
+        <v>3</v>
+      </c>
+      <c r="I34" s="13"/>
+    </row>
+    <row r="35" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G35" s="13">
+        <v>33</v>
+      </c>
+      <c r="H35" s="13">
+        <v>4</v>
+      </c>
+      <c r="I35" s="13"/>
+    </row>
+    <row r="36" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G36" s="13">
+        <v>33</v>
+      </c>
+      <c r="H36" s="13">
+        <v>5</v>
+      </c>
+      <c r="I36" s="13"/>
+    </row>
+    <row r="37" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G37" s="13">
+        <v>34</v>
+      </c>
+      <c r="H37" s="13">
+        <v>2</v>
+      </c>
+      <c r="I37" s="13"/>
+    </row>
+    <row r="38" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G38" s="13">
+        <v>34</v>
+      </c>
+      <c r="H38" s="13">
+        <v>3</v>
+      </c>
+      <c r="I38" s="13"/>
+    </row>
+    <row r="39" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G39" s="13">
+        <v>34</v>
+      </c>
+      <c r="H39" s="13">
+        <v>4</v>
+      </c>
+      <c r="I39" s="13"/>
+    </row>
+    <row r="40" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G40" s="13">
+        <v>34</v>
+      </c>
+      <c r="H40" s="13">
+        <v>5</v>
+      </c>
+      <c r="I40" s="13"/>
+    </row>
+    <row r="41" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G41" s="13">
+        <v>16</v>
+      </c>
+      <c r="H41" s="13">
+        <v>2</v>
+      </c>
+      <c r="I41" s="13"/>
+    </row>
+    <row r="42" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G42" s="13">
+        <v>16</v>
+      </c>
+      <c r="H42" s="13">
+        <v>3</v>
+      </c>
+      <c r="I42" s="13"/>
+    </row>
+    <row r="43" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G43" s="13">
+        <v>16</v>
+      </c>
+      <c r="H43" s="13">
+        <v>4</v>
+      </c>
+      <c r="I43" s="13"/>
+    </row>
+    <row r="44" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G44" s="13">
+        <v>16</v>
+      </c>
+      <c r="H44" s="13">
+        <v>5</v>
+      </c>
+      <c r="I44" s="13"/>
+    </row>
+    <row r="45" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G45" s="13">
+        <v>17</v>
+      </c>
+      <c r="H45" s="13">
+        <v>2</v>
+      </c>
+      <c r="I45" s="13"/>
+    </row>
+    <row r="46" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G46" s="13">
+        <v>17</v>
+      </c>
+      <c r="H46" s="13">
+        <v>3</v>
+      </c>
+      <c r="I46" s="13"/>
+    </row>
+    <row r="47" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G47" s="13">
+        <v>17</v>
+      </c>
+      <c r="H47" s="13">
+        <v>4</v>
+      </c>
+      <c r="I47" s="13"/>
+    </row>
+    <row r="48" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G48" s="13">
+        <v>17</v>
+      </c>
+      <c r="H48" s="13">
+        <v>5</v>
+      </c>
+      <c r="I48" s="13"/>
+    </row>
+    <row r="49" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G49" s="13">
+        <v>18</v>
+      </c>
+      <c r="H49" s="13">
+        <v>2</v>
+      </c>
+      <c r="I49" s="13"/>
+    </row>
+    <row r="50" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G50" s="13">
+        <v>18</v>
+      </c>
+      <c r="H50" s="13">
+        <v>3</v>
+      </c>
+      <c r="I50" s="13"/>
+    </row>
+    <row r="51" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G51" s="13">
+        <v>18</v>
+      </c>
+      <c r="H51" s="13">
+        <v>4</v>
+      </c>
+      <c r="I51" s="13"/>
+    </row>
+    <row r="52" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G52" s="13">
+        <v>18</v>
+      </c>
+      <c r="H52" s="13">
+        <v>5</v>
+      </c>
+      <c r="I52" s="13"/>
+    </row>
+    <row r="53" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G53" s="13">
+        <v>8</v>
+      </c>
+      <c r="H53" s="13">
+        <v>2</v>
+      </c>
+      <c r="I53" s="13"/>
+    </row>
+    <row r="54" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G54" s="13">
+        <v>8</v>
+      </c>
+      <c r="H54" s="13">
+        <v>3</v>
+      </c>
+      <c r="I54" s="13"/>
+    </row>
+    <row r="55" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G55" s="13">
+        <v>8</v>
+      </c>
+      <c r="H55" s="13">
+        <v>4</v>
+      </c>
+      <c r="I55" s="13"/>
+    </row>
+    <row r="56" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G56" s="13">
+        <v>8</v>
+      </c>
+      <c r="H56" s="13">
+        <v>5</v>
+      </c>
+      <c r="I56" s="13"/>
+    </row>
+    <row r="57" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G57" s="13">
+        <v>9</v>
+      </c>
+      <c r="H57" s="13">
+        <v>2</v>
+      </c>
+      <c r="I57" s="13"/>
+    </row>
+    <row r="58" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G58" s="13">
+        <v>9</v>
+      </c>
+      <c r="H58" s="13">
+        <v>3</v>
+      </c>
+      <c r="I58" s="13"/>
+    </row>
+    <row r="59" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G59" s="13">
+        <v>9</v>
+      </c>
+      <c r="H59" s="13">
+        <v>4</v>
+      </c>
+      <c r="I59" s="13"/>
+    </row>
+    <row r="60" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G60" s="13">
+        <v>9</v>
+      </c>
+      <c r="H60" s="13">
+        <v>5</v>
+      </c>
+      <c r="I60" s="13"/>
+    </row>
+    <row r="61" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G61" s="13">
+        <v>10</v>
+      </c>
+      <c r="H61" s="13">
+        <v>2</v>
+      </c>
+      <c r="I61" s="13"/>
+    </row>
+    <row r="62" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G62" s="13">
+        <v>10</v>
+      </c>
+      <c r="H62" s="13">
+        <v>3</v>
+      </c>
+      <c r="I62" s="13"/>
+    </row>
+    <row r="63" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G63" s="13">
+        <v>10</v>
+      </c>
+      <c r="H63" s="13">
+        <v>4</v>
+      </c>
+      <c r="I63" s="13"/>
+    </row>
+    <row r="64" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G64" s="13">
+        <v>10</v>
+      </c>
+      <c r="H64" s="13">
+        <v>5</v>
+      </c>
+      <c r="I64" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="G3:I3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I181"/>
-  <sheetFormatPr defaultColWidth="8.66363636363636" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
     <col min="2" max="4" width="10" style="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="18" style="1" customWidth="1"/>
     <col min="7" max="7" width="24" style="1" customWidth="1"/>
-    <col min="8" max="8" width="31.4454545454545" style="1" customWidth="1"/>
+    <col min="8" max="8" width="31.44140625" style="1" customWidth="1"/>
     <col min="9" max="9" width="12" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.66363636363636" style="1"/>
+    <col min="10" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:9">
+    <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>11</v>
       </c>
@@ -3945,7 +3974,7 @@
       </c>
       <c r="I1" s="10"/>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>128</v>
       </c>
@@ -3974,7 +4003,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>128</v>
       </c>
@@ -4003,7 +4032,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>128</v>
       </c>
@@ -4032,7 +4061,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>128</v>
       </c>
@@ -4061,7 +4090,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>128</v>
       </c>
@@ -4083,7 +4112,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>128</v>
       </c>
@@ -4108,7 +4137,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>128</v>
       </c>
@@ -4133,7 +4162,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>128</v>
       </c>
@@ -4158,7 +4187,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>128</v>
       </c>
@@ -4183,7 +4212,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>128</v>
       </c>
@@ -4205,7 +4234,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>128</v>
       </c>
@@ -4227,7 +4256,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>128</v>
       </c>
@@ -4250,7 +4279,7 @@
       </c>
       <c r="H13" s="9"/>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>128</v>
       </c>
@@ -4272,7 +4301,7 @@
         <v>39.6666666666667</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>128</v>
       </c>
@@ -4294,7 +4323,7 @@
         <v>60.5</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>128</v>
       </c>
@@ -4317,7 +4346,7 @@
       </c>
       <c r="H16" s="9"/>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>128</v>
       </c>
@@ -4339,7 +4368,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>128</v>
       </c>
@@ -4361,7 +4390,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>128</v>
       </c>
@@ -4383,7 +4412,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>128</v>
       </c>
@@ -4405,7 +4434,7 @@
         <v>40.3333333333333</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>128</v>
       </c>
@@ -4427,7 +4456,7 @@
         <v>61.5</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>128</v>
       </c>
@@ -4449,7 +4478,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>128</v>
       </c>
@@ -4471,7 +4500,7 @@
         <v>40.6666666666667</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>128</v>
       </c>
@@ -4493,7 +4522,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
         <v>128</v>
       </c>
@@ -4515,7 +4544,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>128</v>
       </c>
@@ -4537,7 +4566,7 @@
         <v>40.3333333333333</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>128</v>
       </c>
@@ -4559,7 +4588,7 @@
         <v>61.5</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>128</v>
       </c>
@@ -4581,7 +4610,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
         <v>128</v>
       </c>
@@ -4603,7 +4632,7 @@
         <v>40.6666666666667</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>128</v>
       </c>
@@ -4625,7 +4654,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
         <v>128</v>
       </c>
@@ -4647,7 +4676,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>128</v>
       </c>
@@ -4669,7 +4698,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>128</v>
       </c>
@@ -4691,7 +4720,7 @@
         <v>62.5</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>128</v>
       </c>
@@ -4713,7 +4742,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
         <v>128</v>
       </c>
@@ -4735,7 +4764,7 @@
         <v>41.3333333333333</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>128</v>
       </c>
@@ -4757,7 +4786,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
         <v>128</v>
       </c>
@@ -4779,7 +4808,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>64</v>
       </c>
@@ -4801,7 +4830,7 @@
         <v>17.6666666666667</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
         <v>64</v>
       </c>
@@ -4823,7 +4852,7 @@
         <v>27.5</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>64</v>
       </c>
@@ -4845,7 +4874,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="4">
         <v>64</v>
       </c>
@@ -4867,7 +4896,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>64</v>
       </c>
@@ -4889,7 +4918,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
         <v>64</v>
       </c>
@@ -4911,7 +4940,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>64</v>
       </c>
@@ -4933,7 +4962,7 @@
         <v>18.3333333333333</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
         <v>64</v>
       </c>
@@ -4955,7 +4984,7 @@
         <v>28.5</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
         <v>64</v>
       </c>
@@ -4977,7 +5006,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
         <v>64</v>
       </c>
@@ -4999,7 +5028,7 @@
         <v>18.6666666666667</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="4">
         <v>64</v>
       </c>
@@ -5021,7 +5050,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
         <v>64</v>
       </c>
@@ -5043,7 +5072,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
         <v>64</v>
       </c>
@@ -5065,7 +5094,7 @@
         <v>18.3333333333333</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
         <v>64</v>
       </c>
@@ -5087,7 +5116,7 @@
         <v>28.5</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="4">
         <v>64</v>
       </c>
@@ -5109,7 +5138,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="4">
         <v>64</v>
       </c>
@@ -5131,7 +5160,7 @@
         <v>18.6666666666667</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="4">
         <v>64</v>
       </c>
@@ -5153,7 +5182,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="4">
         <v>64</v>
       </c>
@@ -5175,7 +5204,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="4">
         <v>64</v>
       </c>
@@ -5197,7 +5226,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="4">
         <v>64</v>
       </c>
@@ -5219,7 +5248,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="4">
         <v>64</v>
       </c>
@@ -5241,7 +5270,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="4">
         <v>64</v>
       </c>
@@ -5263,7 +5292,7 @@
         <v>19.3333333333333</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="4">
         <v>64</v>
       </c>
@@ -5285,7 +5314,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="4">
         <v>64</v>
       </c>
@@ -5307,7 +5336,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="4">
         <v>64</v>
       </c>
@@ -5329,7 +5358,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="4">
         <v>64</v>
       </c>
@@ -5351,7 +5380,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="4">
         <v>64</v>
       </c>
@@ -5373,7 +5402,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="4">
         <v>64</v>
       </c>
@@ -5395,7 +5424,7 @@
         <v>19.3333333333333</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="4">
         <v>64</v>
       </c>
@@ -5417,7 +5446,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="4">
         <v>64</v>
       </c>
@@ -5439,7 +5468,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="4">
         <v>64</v>
       </c>
@@ -5461,7 +5490,7 @@
         <v>19.6666666666667</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="4">
         <v>64</v>
       </c>
@@ -5483,7 +5512,7 @@
         <v>30.5</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="4">
         <v>64</v>
       </c>
@@ -5505,7 +5534,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="4">
         <v>64</v>
       </c>
@@ -5527,7 +5556,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="4">
         <v>64</v>
       </c>
@@ -5549,7 +5578,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="4">
         <v>64</v>
       </c>
@@ -5571,7 +5600,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="4">
         <v>32</v>
       </c>
@@ -5593,7 +5622,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="4">
         <v>32</v>
       </c>
@@ -5615,7 +5644,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="4">
         <v>32</v>
       </c>
@@ -5637,7 +5666,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="4">
         <v>32</v>
       </c>
@@ -5656,10 +5685,10 @@
       </c>
       <c r="F77" s="6">
         <f t="shared" si="5"/>
-        <v>7.33333333333333</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6">
+        <v>7.3333333333333304</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="4">
         <v>32</v>
       </c>
@@ -5681,7 +5710,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="4">
         <v>32</v>
       </c>
@@ -5703,7 +5732,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="4">
         <v>32</v>
       </c>
@@ -5722,10 +5751,10 @@
       </c>
       <c r="F80" s="6">
         <f t="shared" si="5"/>
-        <v>7.66666666666667</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6">
+        <v>7.6666666666666696</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="4">
         <v>32</v>
       </c>
@@ -5747,7 +5776,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="4">
         <v>32</v>
       </c>
@@ -5769,7 +5798,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="4">
         <v>32</v>
       </c>
@@ -5791,7 +5820,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="4">
         <v>32</v>
       </c>
@@ -5813,7 +5842,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="4">
         <v>32</v>
       </c>
@@ -5835,7 +5864,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="4">
         <v>32</v>
       </c>
@@ -5854,10 +5883,10 @@
       </c>
       <c r="F86" s="6">
         <f t="shared" si="5"/>
-        <v>7.66666666666667</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6">
+        <v>7.6666666666666696</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="4">
         <v>32</v>
       </c>
@@ -5879,7 +5908,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="4">
         <v>32</v>
       </c>
@@ -5901,7 +5930,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="4">
         <v>32</v>
       </c>
@@ -5923,7 +5952,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="4">
         <v>32</v>
       </c>
@@ -5945,7 +5974,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="4">
         <v>32</v>
       </c>
@@ -5967,7 +5996,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="4">
         <v>32</v>
       </c>
@@ -5986,10 +6015,10 @@
       </c>
       <c r="F92" s="6">
         <f t="shared" si="5"/>
-        <v>8.33333333333333</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6">
+        <v>8.3333333333333304</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="4">
         <v>32</v>
       </c>
@@ -6011,7 +6040,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="4">
         <v>32</v>
       </c>
@@ -6033,7 +6062,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="4">
         <v>32</v>
       </c>
@@ -6052,10 +6081,10 @@
       </c>
       <c r="F95" s="6">
         <f t="shared" si="5"/>
-        <v>8.66666666666667</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6">
+        <v>8.6666666666666696</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="4">
         <v>32</v>
       </c>
@@ -6077,7 +6106,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="4">
         <v>32</v>
       </c>
@@ -6099,7 +6128,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="4">
         <v>32</v>
       </c>
@@ -6118,10 +6147,10 @@
       </c>
       <c r="F98" s="6">
         <f t="shared" ref="F98:F129" si="7">((A98+2*B98-C98)/D98)+1-3</f>
-        <v>8.33333333333333</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6">
+        <v>8.3333333333333304</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="4">
         <v>32</v>
       </c>
@@ -6143,7 +6172,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="100" spans="1:6">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="4">
         <v>32</v>
       </c>
@@ -6165,7 +6194,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="101" spans="1:6">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="4">
         <v>32</v>
       </c>
@@ -6184,10 +6213,10 @@
       </c>
       <c r="F101" s="6">
         <f t="shared" si="7"/>
-        <v>8.66666666666667</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6">
+        <v>8.6666666666666696</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="4">
         <v>32</v>
       </c>
@@ -6209,7 +6238,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="103" spans="1:6">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="4">
         <v>32</v>
       </c>
@@ -6231,7 +6260,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="4">
         <v>32</v>
       </c>
@@ -6253,7 +6282,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:6">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="4">
         <v>32</v>
       </c>
@@ -6275,7 +6304,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="4">
         <v>32</v>
       </c>
@@ -6297,7 +6326,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="4">
         <v>32</v>
       </c>
@@ -6316,10 +6345,10 @@
       </c>
       <c r="F107" s="6">
         <f t="shared" si="7"/>
-        <v>9.33333333333333</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6">
+        <v>9.3333333333333304</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="4">
         <v>32</v>
       </c>
@@ -6341,7 +6370,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="109" spans="1:6">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="4">
         <v>32</v>
       </c>
@@ -6363,7 +6392,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="4">
         <v>16</v>
       </c>
@@ -6382,10 +6411,10 @@
       </c>
       <c r="F110" s="6">
         <f t="shared" si="7"/>
-        <v>1.66666666666667</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6">
+        <v>1.6666666666666701</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="4">
         <v>16</v>
       </c>
@@ -6407,7 +6436,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="4">
         <v>16</v>
       </c>
@@ -6429,7 +6458,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="1:6">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="4">
         <v>16</v>
       </c>
@@ -6451,7 +6480,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="114" spans="1:6">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="4">
         <v>16</v>
       </c>
@@ -6473,7 +6502,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:6">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="4">
         <v>16</v>
       </c>
@@ -6495,7 +6524,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" spans="1:6">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="4">
         <v>16</v>
       </c>
@@ -6514,10 +6543,10 @@
       </c>
       <c r="F116" s="6">
         <f t="shared" si="7"/>
-        <v>2.33333333333333</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6">
+        <v>2.3333333333333299</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="4">
         <v>16</v>
       </c>
@@ -6539,7 +6568,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="118" spans="1:6">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="4">
         <v>16</v>
       </c>
@@ -6561,7 +6590,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="119" spans="1:6">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="4">
         <v>16</v>
       </c>
@@ -6580,10 +6609,10 @@
       </c>
       <c r="F119" s="6">
         <f t="shared" si="7"/>
-        <v>2.66666666666667</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6">
+        <v>2.6666666666666701</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="4">
         <v>16</v>
       </c>
@@ -6605,7 +6634,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:6">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="4">
         <v>16</v>
       </c>
@@ -6627,7 +6656,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="122" spans="1:6">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="4">
         <v>16</v>
       </c>
@@ -6646,10 +6675,10 @@
       </c>
       <c r="F122" s="6">
         <f t="shared" si="7"/>
-        <v>2.33333333333333</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6">
+        <v>2.3333333333333299</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="4">
         <v>16</v>
       </c>
@@ -6671,7 +6700,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="124" spans="1:6">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="4">
         <v>16</v>
       </c>
@@ -6693,7 +6722,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:6">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="4">
         <v>16</v>
       </c>
@@ -6712,10 +6741,10 @@
       </c>
       <c r="F125" s="6">
         <f t="shared" si="7"/>
-        <v>2.66666666666667</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6">
+        <v>2.6666666666666701</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="4">
         <v>16</v>
       </c>
@@ -6737,7 +6766,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="127" spans="1:6">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="4">
         <v>16</v>
       </c>
@@ -6759,7 +6788,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="128" spans="1:6">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="4">
         <v>16</v>
       </c>
@@ -6781,7 +6810,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="129" spans="1:6">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="4">
         <v>16</v>
       </c>
@@ -6803,7 +6832,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="130" spans="1:6">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="4">
         <v>16</v>
       </c>
@@ -6825,7 +6854,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="131" spans="1:6">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="4">
         <v>16</v>
       </c>
@@ -6844,10 +6873,10 @@
       </c>
       <c r="F131" s="6">
         <f t="shared" si="9"/>
-        <v>3.33333333333333</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6">
+        <v>3.3333333333333299</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="4">
         <v>16</v>
       </c>
@@ -6869,7 +6898,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="133" spans="1:6">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="4">
         <v>16</v>
       </c>
@@ -6891,7 +6920,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="134" spans="1:6">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="4">
         <v>16</v>
       </c>
@@ -6913,7 +6942,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="135" spans="1:6">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="4">
         <v>16</v>
       </c>
@@ -6935,7 +6964,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="136" spans="1:6">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="4">
         <v>16</v>
       </c>
@@ -6957,7 +6986,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="137" spans="1:6">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="4">
         <v>16</v>
       </c>
@@ -6976,10 +7005,10 @@
       </c>
       <c r="F137" s="6">
         <f t="shared" si="9"/>
-        <v>3.33333333333333</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6">
+        <v>3.3333333333333299</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="4">
         <v>16</v>
       </c>
@@ -7001,7 +7030,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="139" spans="1:6">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="4">
         <v>16</v>
       </c>
@@ -7023,7 +7052,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="140" spans="1:6">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="4">
         <v>16</v>
       </c>
@@ -7042,10 +7071,10 @@
       </c>
       <c r="F140" s="6">
         <f t="shared" si="9"/>
-        <v>3.66666666666667</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6">
+        <v>3.6666666666666701</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="4">
         <v>16</v>
       </c>
@@ -7067,7 +7096,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="142" spans="1:6">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="4">
         <v>16</v>
       </c>
@@ -7089,7 +7118,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="143" spans="1:6">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="4">
         <v>16</v>
       </c>
@@ -7111,7 +7140,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="144" spans="1:6">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="4">
         <v>16</v>
       </c>
@@ -7133,7 +7162,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="145" spans="1:6">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="4">
         <v>16</v>
       </c>
@@ -7155,7 +7184,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="146" spans="1:6">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="4">
         <v>8</v>
       </c>
@@ -7177,7 +7206,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="147" spans="1:6">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="4">
         <v>8</v>
       </c>
@@ -7199,7 +7228,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="148" spans="1:6">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="4">
         <v>8</v>
       </c>
@@ -7221,7 +7250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:6">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="4">
         <v>8</v>
       </c>
@@ -7240,10 +7269,10 @@
       </c>
       <c r="F149" s="6">
         <f t="shared" si="9"/>
-        <v>-0.666666666666667</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6">
+        <v>-0.66666666666666696</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="4">
         <v>8</v>
       </c>
@@ -7265,7 +7294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:6">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="4">
         <v>8</v>
       </c>
@@ -7287,7 +7316,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="152" spans="1:6">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="4">
         <v>8</v>
       </c>
@@ -7306,10 +7335,10 @@
       </c>
       <c r="F152" s="6">
         <f t="shared" si="9"/>
-        <v>-0.333333333333333</v>
-      </c>
-    </row>
-    <row r="153" spans="1:6">
+        <v>-0.33333333333333298</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="4">
         <v>8</v>
       </c>
@@ -7331,7 +7360,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="154" spans="1:6">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="4">
         <v>8</v>
       </c>
@@ -7353,7 +7382,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="155" spans="1:6">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="4">
         <v>8</v>
       </c>
@@ -7375,7 +7404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:6">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="4">
         <v>8</v>
       </c>
@@ -7397,7 +7426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:6">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="4">
         <v>8</v>
       </c>
@@ -7419,7 +7448,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="158" spans="1:6">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="4">
         <v>8</v>
       </c>
@@ -7438,10 +7467,10 @@
       </c>
       <c r="F158" s="6">
         <f t="shared" si="9"/>
-        <v>-0.333333333333333</v>
-      </c>
-    </row>
-    <row r="159" spans="1:6">
+        <v>-0.33333333333333298</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="4">
         <v>8</v>
       </c>
@@ -7463,7 +7492,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="160" spans="1:6">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="4">
         <v>8</v>
       </c>
@@ -7485,7 +7514,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="161" spans="1:6">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="4">
         <v>8</v>
       </c>
@@ -7507,7 +7536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:6">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="4">
         <v>8</v>
       </c>
@@ -7521,7 +7550,7 @@
         <v>2</v>
       </c>
       <c r="E162" s="5">
-        <f t="shared" ref="E162:E193" si="10">TRUNC((A162+2*B162-C162)/D162)+1-3</f>
+        <f t="shared" ref="E162:E181" si="10">TRUNC((A162+2*B162-C162)/D162)+1-3</f>
         <v>1</v>
       </c>
       <c r="F162" s="6">
@@ -7529,7 +7558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:6">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="4">
         <v>8</v>
       </c>
@@ -7551,7 +7580,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="164" spans="1:6">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="4">
         <v>8</v>
       </c>
@@ -7570,10 +7599,10 @@
       </c>
       <c r="F164" s="6">
         <f t="shared" si="11"/>
-        <v>0.333333333333333</v>
-      </c>
-    </row>
-    <row r="165" spans="1:6">
+        <v>0.33333333333333298</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="4">
         <v>8</v>
       </c>
@@ -7595,7 +7624,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="166" spans="1:6">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="4">
         <v>8</v>
       </c>
@@ -7617,7 +7646,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="167" spans="1:6">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" s="4">
         <v>8</v>
       </c>
@@ -7636,10 +7665,10 @@
       </c>
       <c r="F167" s="6">
         <f t="shared" si="11"/>
-        <v>0.666666666666667</v>
-      </c>
-    </row>
-    <row r="168" spans="1:6">
+        <v>0.66666666666666696</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" s="4">
         <v>8</v>
       </c>
@@ -7661,7 +7690,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="169" spans="1:6">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" s="4">
         <v>8</v>
       </c>
@@ -7683,7 +7712,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="170" spans="1:6">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" s="4">
         <v>8</v>
       </c>
@@ -7702,10 +7731,10 @@
       </c>
       <c r="F170" s="6">
         <f t="shared" si="11"/>
-        <v>0.333333333333333</v>
-      </c>
-    </row>
-    <row r="171" spans="1:6">
+        <v>0.33333333333333298</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" s="4">
         <v>8</v>
       </c>
@@ -7727,7 +7756,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="172" spans="1:6">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" s="4">
         <v>8</v>
       </c>
@@ -7749,7 +7778,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="173" spans="1:6">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173" s="4">
         <v>8</v>
       </c>
@@ -7768,10 +7797,10 @@
       </c>
       <c r="F173" s="6">
         <f t="shared" si="11"/>
-        <v>0.666666666666667</v>
-      </c>
-    </row>
-    <row r="174" spans="1:6">
+        <v>0.66666666666666696</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174" s="4">
         <v>8</v>
       </c>
@@ -7793,7 +7822,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="175" spans="1:6">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" s="4">
         <v>8</v>
       </c>
@@ -7815,7 +7844,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="176" spans="1:6">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" s="4">
         <v>8</v>
       </c>
@@ -7837,7 +7866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:6">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" s="4">
         <v>8</v>
       </c>
@@ -7859,7 +7888,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="178" spans="1:6">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" s="4">
         <v>8</v>
       </c>
@@ -7881,7 +7910,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="179" spans="1:6">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" s="4">
         <v>8</v>
       </c>
@@ -7900,10 +7929,10 @@
       </c>
       <c r="F179" s="6">
         <f t="shared" si="11"/>
-        <v>1.33333333333333</v>
-      </c>
-    </row>
-    <row r="180" spans="1:6">
+        <v>1.3333333333333299</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" s="4">
         <v>8</v>
       </c>
@@ -7925,7 +7954,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="181" spans="1:6">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" s="4">
         <v>8</v>
       </c>
@@ -7948,12 +7977,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:F181" etc:filterBottomFollowUsedRange="0">
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="A1:F181" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter/>
-  <legacyDrawing r:id="rId2"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>